<commit_message>
feat: implement Light/Dark mode switcher, mobile compatibility styles, and high contrast visibility fixes
</commit_message>
<xml_diff>
--- a/lead-enquiries.xlsx
+++ b/lead-enquiries.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P8"/>
+  <dimension ref="A1:P9"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -799,9 +799,59 @@
         <v>2026-07-27T12:27:36.379Z</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>LEAD-1003</v>
+      </c>
+      <c r="B9" t="str">
+        <v>gghj</v>
+      </c>
+      <c r="C9" t="str">
+        <v>ddd</v>
+      </c>
+      <c r="D9" t="str">
+        <v>company@google.com</v>
+      </c>
+      <c r="E9" t="str">
+        <v>9999999999</v>
+      </c>
+      <c r="F9">
+        <v>50</v>
+      </c>
+      <c r="G9">
+        <v>1500</v>
+      </c>
+      <c r="H9" t="str">
+        <v>Diwali Gifting</v>
+      </c>
+      <c r="I9" t="str">
+        <v>Download Hub</v>
+      </c>
+      <c r="J9" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="K9" t="str">
+        <v>Catalogue Request</v>
+      </c>
+      <c r="L9" t="str">
+        <v>Suspicious</v>
+      </c>
+      <c r="M9" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="N9" t="str">
+        <v>Duplicate inquiry phone within 24h</v>
+      </c>
+      <c r="O9" t="str">
+        <v/>
+      </c>
+      <c r="P9" t="str">
+        <v>2026-07-28T11:15:06.220Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P9"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>